<commit_message>
gemini + gpt autograded
</commit_message>
<xml_diff>
--- a/Automatic Bread Maker/Grading/2 stage/6-examples/Automatic-Bread-Maker_Grading_2-stage_2026-03-12_6-examples_Gemini3.1ProPreviewGeneration_GPT5.5AutoGrading.xlsx
+++ b/Automatic Bread Maker/Grading/2 stage/6-examples/Automatic-Bread-Maker_Grading_2-stage_2026-03-12_6-examples_Gemini3.1ProPreviewGeneration_GPT5.5AutoGrading.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="17720" yWindow="-21000" windowWidth="30240" windowHeight="17300" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Automatic Bread Maker" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gemini Generation" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metrics" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Automatic Bread Maker" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="GPT-5.5 Grading" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Metrics" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -6061,7 +6061,7 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>GPT-5 Generation</t>
+          <t>Grading</t>
         </is>
       </c>
       <c r="D1" s="15" t="inlineStr">
@@ -6086,7 +6086,7 @@
       </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
-          <t>Initial state correctly transitions to Off</t>
+          <t>Initial pseudostate enters Off.</t>
         </is>
       </c>
     </row>
@@ -6106,7 +6106,7 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Off state is present</t>
+          <t>Off state is explicitly modeled.</t>
         </is>
       </c>
     </row>
@@ -6126,7 +6126,7 @@
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>Transition powerOn from Off to On is present</t>
+          <t>Off transitions to On using turnOn which is equivalent.</t>
         </is>
       </c>
     </row>
@@ -6146,7 +6146,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>On composite state is present</t>
+          <t>On is modeled as a composite state containing operating behavior.</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D6" s="21" t="inlineStr">
         <is>
-          <t>Transition powerOff from On to Off is present</t>
+          <t>On transitions to Off using turnOff which is equivalent.</t>
         </is>
       </c>
       <c r="E6" s="6" t="n"/>
@@ -6204,7 +6204,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Setup composite state is present</t>
+          <t>Setup composite state is explicitly modeled.</t>
         </is>
       </c>
     </row>
@@ -6224,7 +6224,7 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Medium is the initial state in CrustSelection region</t>
+          <t>Crust selection initializes to Medium within Setup.</t>
         </is>
       </c>
     </row>
@@ -6240,11 +6240,11 @@
         </is>
       </c>
       <c r="C9" s="5" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>initializeDefaults() action is present but not explicitly showing delay=0 and selectFirstCourse() separately</t>
+          <t>Setup entry sets timer to 0 and selects course 1.</t>
         </is>
       </c>
     </row>
@@ -6264,7 +6264,7 @@
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Medium state is present in CrustSelection region</t>
+          <t>Medium crust state is present.</t>
         </is>
       </c>
     </row>
@@ -6284,7 +6284,7 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Initial transition to Medium is present</t>
+          <t>Initial transition in crust selection targets Medium.</t>
         </is>
       </c>
     </row>
@@ -6304,7 +6304,7 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Transition from Medium to Dark on crust event is present</t>
+          <t>Crust button moves Medium to Dark.</t>
         </is>
       </c>
     </row>
@@ -6324,7 +6324,7 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Dark state is present</t>
+          <t>Dark crust state is present.</t>
         </is>
       </c>
     </row>
@@ -6344,7 +6344,7 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Transition from Dark to Light on crust event is present</t>
+          <t>Crust button moves Dark to Light.</t>
         </is>
       </c>
     </row>
@@ -6364,7 +6364,7 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Light state is present</t>
+          <t>Light crust state is present.</t>
         </is>
       </c>
     </row>
@@ -6380,11 +6380,11 @@
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>No history state is present; menu transitions stay within CourseSelected state</t>
+          <t>Equivalent preservation is handled by concurrent setup regions rather than an explicit history state.</t>
         </is>
       </c>
     </row>
@@ -6400,11 +6400,11 @@
         </is>
       </c>
       <c r="C17" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>No transition to history state; menu handled within CourseSelected</t>
+          <t>Menu is modeled as a course selection self transition preserving other setup choices.</t>
         </is>
       </c>
     </row>
@@ -6424,7 +6424,7 @@
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>selectNextCourse() action is present on menu transition</t>
+          <t>Menu action nextCourse captures selecting the next course.</t>
         </is>
       </c>
       <c r="E18" s="6" t="n"/>
@@ -6462,7 +6462,7 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Plus transitions within Setup are present</t>
+          <t>Plus is modeled as a self transition within timer setup.</t>
         </is>
       </c>
     </row>
@@ -6482,7 +6482,7 @@
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>Guard [timer &lt; 18h] is semantically equivalent to delay &lt;= 17*60+50</t>
+          <t>Guard timer &lt; 18h correctly permits increments up to 18 hours.</t>
         </is>
       </c>
     </row>
@@ -6502,7 +6502,7 @@
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>increaseTimer(10min) action is semantically equivalent</t>
+          <t>increaseTimer by 10 minutes is modeled.</t>
         </is>
       </c>
     </row>
@@ -6522,7 +6522,7 @@
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>Minus transitions within Setup are present</t>
+          <t>Minus is modeled as a self transition within timer setup.</t>
         </is>
       </c>
     </row>
@@ -6542,7 +6542,7 @@
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Guard [timer &gt; 10min] is semantically equivalent to delay &gt;= 10</t>
+          <t>Guard timer &gt; 0 is equivalent because the timer changes in 10 minute steps.</t>
         </is>
       </c>
     </row>
@@ -6562,7 +6562,7 @@
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>decreaseTimer(10min) action is semantically equivalent</t>
+          <t>decreaseTimer by 10 minutes is modeled.</t>
         </is>
       </c>
       <c r="E24" s="6" t="n"/>
@@ -6600,7 +6600,7 @@
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Transition from Setup to Countdown with guard [timer &gt; 0] is present</t>
+          <t>Start with timer greater than 0 goes to Countdown.</t>
         </is>
       </c>
     </row>
@@ -6620,7 +6620,7 @@
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>Guard [timer &gt; 0] is semantically equivalent to delay &gt; 0</t>
+          <t>Guard timer &gt; 0 is present.</t>
         </is>
       </c>
     </row>
@@ -6640,7 +6640,7 @@
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Transition from Setup to BakingProcess with guard [timer == 0] is present</t>
+          <t>Start with timer equal to 0 goes directly to baking process.</t>
         </is>
       </c>
     </row>
@@ -6660,7 +6660,7 @@
       </c>
       <c r="D28" s="8" t="inlineStr">
         <is>
-          <t>Guard [timer == 0] is semantically equivalent to delay == 0</t>
+          <t>Guard timer == 0 is present.</t>
         </is>
       </c>
     </row>
@@ -6680,7 +6680,7 @@
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Countdown state is present</t>
+          <t>Countdown state is explicitly modeled.</t>
         </is>
       </c>
     </row>
@@ -6696,11 +6696,11 @@
         </is>
       </c>
       <c r="C30" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D30" s="8" t="inlineStr">
         <is>
-          <t>clearTimer() action is present; setCourseTimes() is implied in the model flow</t>
+          <t>No action sets course specific phase times before delayed baking.</t>
         </is>
       </c>
     </row>
@@ -6720,7 +6720,7 @@
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Transition from Countdown to BakingProcess on timerElapsed is present</t>
+          <t>Countdown transitions to the baking process when the timer finishes.</t>
         </is>
       </c>
       <c r="E31" s="6" t="n"/>
@@ -6758,7 +6758,7 @@
       </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>Transition from Countdown to Setup on stop is present</t>
+          <t>Stop from Countdown returns to Setup.</t>
         </is>
       </c>
       <c r="E32" s="6" t="n"/>
@@ -6792,11 +6792,11 @@
         </is>
       </c>
       <c r="C33" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>clearTimer() action is present on stop transition</t>
+          <t>No action sets course specific phase times before immediate baking.</t>
         </is>
       </c>
     </row>
@@ -6816,7 +6816,7 @@
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>BakingProcess composite state is present</t>
+          <t>BakingProcess composite represents the baking process.</t>
         </is>
       </c>
     </row>
@@ -6836,7 +6836,7 @@
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Initial state in BakingProcess transitions to Kneading</t>
+          <t>Baking process initial pseudostate enters Kneading.</t>
         </is>
       </c>
     </row>
@@ -6856,7 +6856,7 @@
       </c>
       <c r="D36" s="8" t="inlineStr">
         <is>
-          <t>Kneading state is present</t>
+          <t>Kneading state is present.</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>startKneading() entry action is present</t>
+          <t>Kneading has entry action startKneading.</t>
         </is>
       </c>
     </row>
@@ -6896,7 +6896,7 @@
       </c>
       <c r="D38" s="8" t="inlineStr">
         <is>
-          <t>stopKneading() exit action is present</t>
+          <t>Kneading has exit action stopKneading.</t>
         </is>
       </c>
     </row>
@@ -6916,7 +6916,7 @@
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Initial transition to Kneading is present</t>
+          <t>Initial transition in baking process targets Kneading.</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D40" s="8" t="inlineStr">
         <is>
-          <t>Transition from Kneading to Rising is present</t>
+          <t>Kneading transitions to Rising after kneading time.</t>
         </is>
       </c>
       <c r="E40" s="6" t="n"/>
@@ -6974,7 +6974,7 @@
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Rising state is present</t>
+          <t>Rising state is present.</t>
         </is>
       </c>
       <c r="E41" s="6" t="n"/>
@@ -7012,7 +7012,7 @@
       </c>
       <c r="D42" s="8" t="inlineStr">
         <is>
-          <t>Transition from Rising to Baking is present</t>
+          <t>Rising transitions to Baking after rising time.</t>
         </is>
       </c>
       <c r="E42" s="6" t="n"/>
@@ -7050,7 +7050,7 @@
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>Baking state is present</t>
+          <t>Baking phase state is present.</t>
         </is>
       </c>
       <c r="E43" s="6" t="n"/>
@@ -7088,7 +7088,7 @@
       </c>
       <c r="D44" s="8" t="inlineStr">
         <is>
-          <t>heat() do action is present</t>
+          <t>Baking phase includes heat as do activity.</t>
         </is>
       </c>
       <c r="E44" s="6" t="n"/>
@@ -7126,7 +7126,7 @@
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Transition from Baking to Warming is present</t>
+          <t>Baking transitions to Warming after baking time.</t>
         </is>
       </c>
       <c r="E45" s="6" t="n"/>
@@ -7164,7 +7164,7 @@
       </c>
       <c r="D46" s="8" t="inlineStr">
         <is>
-          <t>Warming state is present</t>
+          <t>Warming state is present.</t>
         </is>
       </c>
       <c r="E46" s="6" t="n"/>
@@ -7202,7 +7202,7 @@
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>warm() do action is present</t>
+          <t>Warming includes warm as do activity.</t>
         </is>
       </c>
       <c r="E47" s="6" t="n"/>
@@ -7240,7 +7240,7 @@
       </c>
       <c r="D48" s="23" t="inlineStr">
         <is>
-          <t>Transition from Warming to Setup after 60min is present</t>
+          <t>Warming returns to Setup after 60 minutes.</t>
         </is>
       </c>
       <c r="E48" s="6" t="n"/>
@@ -7278,7 +7278,7 @@
       </c>
       <c r="D49" s="21" t="inlineStr">
         <is>
-          <t>Transition from BakingProcess to Setup on stop is present</t>
+          <t>Stop from the baking process returns to Setup.</t>
         </is>
       </c>
       <c r="E49" s="6" t="n"/>
@@ -7316,7 +7316,7 @@
       </c>
       <c r="D50" s="26" t="inlineStr">
         <is>
-          <t>No additional incorrect states present</t>
+          <t>No fundamentally incorrect extra states are present.</t>
         </is>
       </c>
       <c r="E50" s="6" t="n"/>
@@ -7354,7 +7354,7 @@
       </c>
       <c r="D51" s="8" t="inlineStr">
         <is>
-          <t>No additional incorrect transitions present</t>
+          <t>No fundamentally incorrect extra transitions are present.</t>
         </is>
       </c>
     </row>
@@ -7374,7 +7374,7 @@
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>No additional incorrect guards present</t>
+          <t>No fundamentally incorrect extra guards are present.</t>
         </is>
       </c>
     </row>
@@ -7394,7 +7394,7 @@
       </c>
       <c r="D53" s="8" t="inlineStr">
         <is>
-          <t>No additional incorrect actions present</t>
+          <t>No fundamentally incorrect extra actions are present.</t>
         </is>
       </c>
     </row>
@@ -7414,7 +7414,7 @@
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>No additional incorrect composite states present</t>
+          <t>Extra composites are reasonable decomposition of setup behavior.</t>
         </is>
       </c>
     </row>
@@ -7434,7 +7434,7 @@
       </c>
       <c r="D55" s="8" t="inlineStr">
         <is>
-          <t>Regions are used appropriately for parallel behavior in Setup</t>
+          <t>Concurrent regions reasonably model simultaneous setup choices.</t>
         </is>
       </c>
     </row>
@@ -7454,7 +7454,7 @@
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>No additional incorrect history states present</t>
+          <t>No incorrect extra history states are present.</t>
         </is>
       </c>
     </row>
@@ -12214,7 +12214,7 @@
     <row r="1" ht="15.75" customHeight="1" s="80">
       <c r="A1" s="84" t="inlineStr">
         <is>
-          <t>Generated by GPT-5</t>
+          <t>Generated by Gemini 3.1 Pro</t>
         </is>
       </c>
       <c r="J1" s="36" t="inlineStr">
@@ -12281,15 +12281,15 @@
         <v/>
       </c>
       <c r="C3" s="41">
-        <f>SUMIF('GPT-5 Generation'!$A$2:$A$49, $A3, 'GPT-5 Generation'!$C$2:$C$49)</f>
+        <f>SUMIF('GPT-5.5 Grading'!$A$2:$A$49, $A3, 'GPT-5.5 Grading'!$C$2:$C$49)</f>
         <v/>
       </c>
       <c r="D3" s="41">
-        <f>SUMIF('GPT-5 Generation'!$A$50:$A$56, $A3, 'GPT-5 Generation'!$C$50:$C$56)</f>
+        <f>SUMIF('GPT-5.5 Grading'!$A$50:$A$56, $A3, 'GPT-5.5 Grading'!$C$50:$C$56)</f>
         <v/>
       </c>
       <c r="E3" s="41">
-        <f>COUNTIFS('GPT-5 Generation'!$A$2:$A$49, $A3, 'GPT-5 Generation'!$C$2:$C$49,0)</f>
+        <f>COUNTIFS('GPT-5.5 Grading'!$A$2:$A$49, $A3, 'GPT-5.5 Grading'!$C$2:$C$49,0)</f>
         <v/>
       </c>
       <c r="F3" s="41">
@@ -12317,15 +12317,15 @@
         <v/>
       </c>
       <c r="C4" s="41">
-        <f>SUMIF('GPT-5 Generation'!$A$2:$A$49, $A4, 'GPT-5 Generation'!$C$2:$C$49)</f>
+        <f>SUMIF('GPT-5.5 Grading'!$A$2:$A$49, $A4, 'GPT-5.5 Grading'!$C$2:$C$49)</f>
         <v/>
       </c>
       <c r="D4" s="41">
-        <f>SUMIF('GPT-5 Generation'!$A$50:$A$56, $A4, 'GPT-5 Generation'!$C$50:$C$56)</f>
+        <f>SUMIF('GPT-5.5 Grading'!$A$50:$A$56, $A4, 'GPT-5.5 Grading'!$C$50:$C$56)</f>
         <v/>
       </c>
       <c r="E4" s="41">
-        <f>COUNTIFS('GPT-5 Generation'!$A$2:$A$49, $A4, 'GPT-5 Generation'!$C$2:$C$49,0)</f>
+        <f>COUNTIFS('GPT-5.5 Grading'!$A$2:$A$49, $A4, 'GPT-5.5 Grading'!$C$2:$C$49,0)</f>
         <v/>
       </c>
       <c r="F4" s="41">
@@ -12357,15 +12357,15 @@
         <v/>
       </c>
       <c r="C5" s="41">
-        <f>SUMIF('GPT-5 Generation'!$A$2:$A$49, $A5, 'GPT-5 Generation'!$C$2:$C$49)</f>
+        <f>SUMIF('GPT-5.5 Grading'!$A$2:$A$49, $A5, 'GPT-5.5 Grading'!$C$2:$C$49)</f>
         <v/>
       </c>
       <c r="D5" s="41">
-        <f>SUMIF('GPT-5 Generation'!$A$50:$A$56, $A5, 'GPT-5 Generation'!$C$50:$C$56)</f>
+        <f>SUMIF('GPT-5.5 Grading'!$A$50:$A$56, $A5, 'GPT-5.5 Grading'!$C$50:$C$56)</f>
         <v/>
       </c>
       <c r="E5" s="41">
-        <f>COUNTIFS('GPT-5 Generation'!$A$2:$A$49, $A5, 'GPT-5 Generation'!$C$2:$C$49,0)</f>
+        <f>COUNTIFS('GPT-5.5 Grading'!$A$2:$A$49, $A5, 'GPT-5.5 Grading'!$C$2:$C$49,0)</f>
         <v/>
       </c>
       <c r="F5" s="41">
@@ -12382,7 +12382,7 @@
       </c>
       <c r="J5" s="44" t="inlineStr">
         <is>
-          <t>GPT-5</t>
+          <t>GPT-5.5</t>
         </is>
       </c>
     </row>
@@ -12397,15 +12397,15 @@
         <v/>
       </c>
       <c r="C6" s="41">
-        <f>SUMIF('GPT-5 Generation'!$A$2:$A$49, $A6, 'GPT-5 Generation'!$C$2:$C$49)</f>
+        <f>SUMIF('GPT-5.5 Grading'!$A$2:$A$49, $A6, 'GPT-5.5 Grading'!$C$2:$C$49)</f>
         <v/>
       </c>
       <c r="D6" s="41">
-        <f>SUMIF('GPT-5 Generation'!$A$50:$A$56, $A6, 'GPT-5 Generation'!$C$50:$C$56)</f>
+        <f>SUMIF('GPT-5.5 Grading'!$A$50:$A$56, $A6, 'GPT-5.5 Grading'!$C$50:$C$56)</f>
         <v/>
       </c>
       <c r="E6" s="41">
-        <f>COUNTIFS('GPT-5 Generation'!$A$2:$A$49, $A6, 'GPT-5 Generation'!$C$2:$C$49,0)</f>
+        <f>COUNTIFS('GPT-5.5 Grading'!$A$2:$A$49, $A6, 'GPT-5.5 Grading'!$C$2:$C$49,0)</f>
         <v/>
       </c>
       <c r="F6" s="41">
@@ -12433,15 +12433,15 @@
         <v/>
       </c>
       <c r="C7" s="41">
-        <f>SUMIF('GPT-5 Generation'!$A$2:$A$49, $A7, 'GPT-5 Generation'!$C$2:$C$49)</f>
+        <f>SUMIF('GPT-5.5 Grading'!$A$2:$A$49, $A7, 'GPT-5.5 Grading'!$C$2:$C$49)</f>
         <v/>
       </c>
       <c r="D7" s="41">
-        <f>SUMIF('GPT-5 Generation'!$A$50:$A$56, $A7, 'GPT-5 Generation'!$C$50:$C$56)</f>
+        <f>SUMIF('GPT-5.5 Grading'!$A$50:$A$56, $A7, 'GPT-5.5 Grading'!$C$50:$C$56)</f>
         <v/>
       </c>
       <c r="E7" s="41">
-        <f>COUNTIFS('GPT-5 Generation'!$A$2:$A$49, $A7, 'GPT-5 Generation'!$C$2:$C$49,0)</f>
+        <f>COUNTIFS('GPT-5.5 Grading'!$A$2:$A$49, $A7, 'GPT-5.5 Grading'!$C$2:$C$49,0)</f>
         <v/>
       </c>
       <c r="F7" s="41">
@@ -12473,15 +12473,15 @@
         <v/>
       </c>
       <c r="C8" s="41">
-        <f>SUMIF('GPT-5 Generation'!$A$2:$A$49, $A8, 'GPT-5 Generation'!$C$2:$C$49)</f>
+        <f>SUMIF('GPT-5.5 Grading'!$A$2:$A$49, $A8, 'GPT-5.5 Grading'!$C$2:$C$49)</f>
         <v/>
       </c>
       <c r="D8" s="41">
-        <f>SUMIF('GPT-5 Generation'!$A$50:$A$56, $A8, 'GPT-5 Generation'!$C$50:$C$56)</f>
+        <f>SUMIF('GPT-5.5 Grading'!$A$50:$A$56, $A8, 'GPT-5.5 Grading'!$C$50:$C$56)</f>
         <v/>
       </c>
       <c r="E8" s="41">
-        <f>COUNTIFS('GPT-5 Generation'!$A$2:$A$49, $A8, 'GPT-5 Generation'!$C$2:$C$49,0)</f>
+        <f>COUNTIFS('GPT-5.5 Grading'!$A$2:$A$49, $A8, 'GPT-5.5 Grading'!$C$2:$C$49,0)</f>
         <v/>
       </c>
       <c r="F8" s="41">
@@ -12498,7 +12498,7 @@
       </c>
       <c r="J8" s="44" t="inlineStr">
         <is>
-          <t>Gemini</t>
+          <t>Gemini 3.1 Pro</t>
         </is>
       </c>
     </row>
@@ -12513,15 +12513,15 @@
         <v/>
       </c>
       <c r="C9" s="41">
-        <f>SUMIF('GPT-5 Generation'!$A$2:$A$49, $A9, 'GPT-5 Generation'!$C$2:$C$49)</f>
+        <f>SUMIF('GPT-5.5 Grading'!$A$2:$A$49, $A9, 'GPT-5.5 Grading'!$C$2:$C$49)</f>
         <v/>
       </c>
       <c r="D9" s="41">
-        <f>SUMIF('GPT-5 Generation'!$A$50:$A$56, $A9, 'GPT-5 Generation'!$C$50:$C$56)</f>
+        <f>SUMIF('GPT-5.5 Grading'!$A$50:$A$56, $A9, 'GPT-5.5 Grading'!$C$50:$C$56)</f>
         <v/>
       </c>
       <c r="E9" s="41">
-        <f>COUNTIFS('GPT-5 Generation'!$A$2:$A$49, $A9, 'GPT-5 Generation'!$C$2:$C$49,0)</f>
+        <f>COUNTIFS('GPT-5.5 Grading'!$A$2:$A$49, $A9, 'GPT-5.5 Grading'!$C$2:$C$49,0)</f>
         <v/>
       </c>
       <c r="F9" s="41">

</xml_diff>